<commit_message>
Flere værker og smårettelser i teksten
</commit_message>
<xml_diff>
--- a/Tekster og billeder til Keramikruten.xlsx
+++ b/Tekster og billeder til Keramikruten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elisabethtejlmand/Documents/GitHub/guide-til-middelfart/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ADC1277-C0A4-4440-8205-9332FFCAEE30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7605A46E-FA7F-9845-B8FA-78692EC70F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8880" yWindow="4360" windowWidth="28240" windowHeight="17240" xr2:uid="{02FFEFA7-C0A6-4249-8E30-DEFBC5A1D164}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="75">
   <si>
     <t>id</t>
   </si>
@@ -222,6 +222,48 @@
   </si>
   <si>
     <t>9.722185</t>
+  </si>
+  <si>
+    <t>livsnyderne</t>
+  </si>
+  <si>
+    <t>Livsnyderne</t>
+  </si>
+  <si>
+    <t>Havnefronten</t>
+  </si>
+  <si>
+    <t>Skal du op og sidde?</t>
+  </si>
+  <si>
+    <t>I vandet omkring Middelfart boltrer en af Danmarks største bestande af hvaler sig; nemlig den lille, legesyge marsvin. Hold godt øje, så ser du sikkert en finne bryde vandoverfladen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Det er svært at vælge det bedste spisested - for smag og behag er forskellig. Guldkronen på Gl. Torv er specialister i den hyggelige atmosfære og dansk smørebrød, mens Cafe Razz er indbegrebet af traditionel cafemad. Længere nede ad Algade finder du skønne spisesteder som perler på en snor. Google Maps kan guide dig. </t>
+  </si>
+  <si>
+    <t>55.506345</t>
+  </si>
+  <si>
+    <t>9.732167</t>
+  </si>
+  <si>
+    <t>Stoflig sanselighed</t>
+  </si>
+  <si>
+    <t>Den dragende dråbe</t>
+  </si>
+  <si>
+    <t>De sidste værker er i parken ved Clay Keramikmuseum</t>
+  </si>
+  <si>
+    <t>Gå gennem Nytorvs port til Havnegade og bevæg dig mod syd langs vandet.</t>
+  </si>
+  <si>
+    <t>• • • https://maps.app.goo.gl/Wqa6YgPdz8Hgc7Zk9?g_st=ic</t>
+  </si>
+  <si>
+    <t>Tag en lille omvej forbi Gl. Havns karakteriske røde værtsbygninger, hvor man har bygget smakkejoller og klinkbygning, der er klasificeret som Verdenskulturarv af UNESCO.</t>
   </si>
 </sst>
 </file>
@@ -297,7 +339,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -312,6 +354,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -656,8 +699,8 @@
     <col min="6" max="6" width="26.33203125" customWidth="1"/>
     <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5" customWidth="1"/>
-    <col min="10" max="10" width="21" customWidth="1"/>
+    <col min="9" max="9" width="17.83203125" customWidth="1"/>
+    <col min="10" max="11" width="21" customWidth="1"/>
     <col min="12" max="12" width="42.83203125" customWidth="1"/>
     <col min="14" max="14" width="48.5" customWidth="1"/>
     <col min="15" max="15" width="33.83203125" customWidth="1"/>
@@ -742,6 +785,9 @@
       <c r="H2" s="9" t="s">
         <v>60</v>
       </c>
+      <c r="I2" t="s">
+        <v>70</v>
+      </c>
       <c r="J2" s="6" t="s">
         <v>40</v>
       </c>
@@ -786,8 +832,14 @@
       <c r="H3" s="9" t="s">
         <v>54</v>
       </c>
+      <c r="I3" t="s">
+        <v>69</v>
+      </c>
       <c r="J3" s="6" t="s">
         <v>41</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>74</v>
       </c>
       <c r="N3" s="6" t="s">
         <v>25</v>
@@ -890,7 +942,9 @@
       <c r="N5" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="3"/>
+      <c r="O5" s="8" t="s">
+        <v>72</v>
+      </c>
       <c r="P5" t="s">
         <v>44</v>
       </c>
@@ -898,22 +952,54 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="17" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
+    <row r="6" spans="1:17" ht="137" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="4">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="3">
+        <v>2001</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>65</v>
+      </c>
       <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
+      <c r="L6" s="8" t="s">
+        <v>66</v>
+      </c>
       <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
+      <c r="N6" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="P6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="7" spans="1:17" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
@@ -1124,6 +1210,7 @@
     <hyperlink ref="N2" r:id="rId1" xr:uid="{425307A9-2A13-124F-A947-E6A946E98065}"/>
     <hyperlink ref="N4" r:id="rId2" xr:uid="{D5DEB3DA-93D1-6C4B-B6EE-A954DA83D819}"/>
     <hyperlink ref="N5" r:id="rId3" xr:uid="{D082706D-F5AF-F445-B8F7-AAB60CDD41FD}"/>
+    <hyperlink ref="N6" r:id="rId4" display="https://maps.app.goo.gl/Wqa6YgPdz8Hgc7Zk9?g_st=ic" xr:uid="{F4BBC5C5-A02A-2A43-86DE-EBFD25438B5E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>